<commit_message>
Clear the fiscal-effect verify note: Abiad et al. (2009) checked
The 1.5 fiscal effect matches Abiad et al. (2009), p. 23, footnote 22
(Table 2, row 1): raising government consumption by 1% of GDP is
associated with a ~1.5 point smaller medium-run (T+7) output loss after
banking crises. Model value unchanged; only the source note is updated.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DQ1ThXX2e9pJJKTMCX3QJe
</commit_message>
<xml_diff>
--- a/capabilities/economic-research/model.xlsx
+++ b/capabilities/economic-research/model.xlsx
@@ -140,9 +140,7 @@
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -515,10 +513,10 @@
   <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" style="2" min="1" max="1"/>
+    <col width="14" customWidth="1" style="2" min="2" max="2"/>
+    <col width="50" customWidth="1" style="2" min="3" max="3"/>
+    <col width="90" customWidth="1" style="2" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -529,7 +527,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Every named input from capabilities/economic-research/spec.md (locked 2026-10-05). Yellow = source value; derived values are formulas at full precision.</t>
         </is>
@@ -913,7 +911,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Abiad et al. (2009) — verify against the PDF before final</t>
+          <t>Abiad et al. (2009), p. 23, fn. 22: +1% of GDP government consumption ≈ 1.5 pt smaller medium-run (T+7) output loss; banking crises; association (verified against the PDF 2026-10-08)</t>
         </is>
       </c>
     </row>
@@ -1215,11 +1213,11 @@
   <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" style="2" min="1" max="1"/>
+    <col width="16" customWidth="1" style="2" min="2" max="2"/>
+    <col width="16" customWidth="1" style="2" min="3" max="3"/>
+    <col width="16" customWidth="1" style="2" min="4" max="4"/>
+    <col width="16" customWidth="1" style="2" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1230,13 +1228,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>BASE_2026 = 100; BASE_t = BASE_{t−1} × (1 + G_t / 100), grown at IMF WEO April 2026 rates.</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1402,12 +1399,12 @@
   <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" style="2" min="1" max="1"/>
+    <col width="20" customWidth="1" style="2" min="2" max="2"/>
+    <col width="20" customWidth="1" style="2" min="3" max="3"/>
+    <col width="22" customWidth="1" style="2" min="4" max="4"/>
+    <col width="20" customWidth="1" style="2" min="5" max="5"/>
+    <col width="20" customWidth="1" style="2" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1418,13 +1415,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>GAP_t = MIN(0, GAP_{t−1} × (1 − BASE_RECOVERY_RATE) + RECOVERY_PTS / 4); SCEN_t = BASE_t × (1 + GAP_t / 100).</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1507,7 +1503,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
@@ -1679,10 +1674,10 @@
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" style="2" min="1" max="1"/>
+    <col width="28" customWidth="1" style="2" min="2" max="2"/>
+    <col width="28" customWidth="1" style="2" min="3" max="3"/>
+    <col width="70" customWidth="1" style="2" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1693,13 +1688,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>RECOVERED_5 = 1 − GAP_2031 / GAP_2027. Falsifier from the brief: if China's RECOVERED_5 ≥ the U.S. RECOVERED_5, the hypothesis is wrong.</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1783,7 +1777,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
@@ -1821,27 +1814,27 @@
   <dimension ref="A1:U33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="13" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="13" customWidth="1" min="19" max="19"/>
-    <col width="13" customWidth="1" min="20" max="20"/>
-    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="46" customWidth="1" style="2" min="1" max="1"/>
+    <col width="13" customWidth="1" style="2" min="2" max="2"/>
+    <col width="13" customWidth="1" style="2" min="3" max="3"/>
+    <col width="13" customWidth="1" style="2" min="4" max="4"/>
+    <col width="13" customWidth="1" style="2" min="5" max="5"/>
+    <col width="13" customWidth="1" style="2" min="6" max="6"/>
+    <col width="13" customWidth="1" style="2" min="7" max="7"/>
+    <col width="13" customWidth="1" style="2" min="8" max="8"/>
+    <col width="13" customWidth="1" style="2" min="9" max="9"/>
+    <col width="13" customWidth="1" style="2" min="10" max="10"/>
+    <col width="13" customWidth="1" style="2" min="11" max="11"/>
+    <col width="13" customWidth="1" style="2" min="12" max="12"/>
+    <col width="13" customWidth="1" style="2" min="13" max="13"/>
+    <col width="13" customWidth="1" style="2" min="14" max="14"/>
+    <col width="13" customWidth="1" style="2" min="15" max="15"/>
+    <col width="13" customWidth="1" style="2" min="16" max="16"/>
+    <col width="13" customWidth="1" style="2" min="17" max="17"/>
+    <col width="13" customWidth="1" style="2" min="18" max="18"/>
+    <col width="13" customWidth="1" style="2" min="19" max="19"/>
+    <col width="13" customWidth="1" style="2" min="20" max="20"/>
+    <col width="13" customWidth="1" style="2" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1852,13 +1845,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Each row reruns the full gap path with its own values. Changed value is shown in the row; other columns reference the named inputs.</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3943,7 +3935,6 @@
         <v/>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
@@ -4024,11 +4015,11 @@
   <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" style="2" min="1" max="1"/>
+    <col width="22" customWidth="1" style="2" min="2" max="2"/>
+    <col width="22" customWidth="1" style="2" min="3" max="3"/>
+    <col width="22" customWidth="1" style="2" min="4" max="4"/>
+    <col width="22" customWidth="1" style="2" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4039,7 +4030,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Expected values are hand calculations typed in as targets. They are not referenced by any calculation on the other sheets.</t>
         </is>

</xml_diff>